<commit_message>
Learning Pivot Table and charts
</commit_message>
<xml_diff>
--- a/Excel/ETL tools/Excel_Text_Functions_LEFT_RIGHT_MID_LEN3.xlsx
+++ b/Excel/ETL tools/Excel_Text_Functions_LEFT_RIGHT_MID_LEN3.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Arbor all Folder\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Arbor all Folder\Excel\ETL tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60F0943B-21EC-4517-AC9F-DDC04733DDE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D034B7A5-29F1-4988-8A99-5D7B4753BE1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{32F7D32F-EBFD-430F-914D-CE2C2076F620}"/>
   </bookViews>
@@ -444,29 +444,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -484,22 +474,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -517,22 +501,6 @@
   </cellStyles>
   <dxfs count="11">
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
@@ -642,26 +610,42 @@
       </border>
     </dxf>
     <dxf>
-      <border>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
         <right style="thin">
           <color indexed="64"/>
         </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
   </dxfs>
@@ -696,15 +680,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{446CC8FA-01E3-483B-8CA2-40098F81BBC1}" name="Customer_Data" displayName="Customer_Data" ref="A1:F11" tableType="queryTable" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0" headerRowBorderDxfId="9" tableBorderDxfId="10" totalsRowBorderDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{446CC8FA-01E3-483B-8CA2-40098F81BBC1}" name="Customer_Data" displayName="Customer_Data" ref="A1:F11" tableType="queryTable" totalsRowShown="0" headerRowDxfId="10" dataDxfId="8" headerRowBorderDxfId="9" tableBorderDxfId="7" totalsRowBorderDxfId="6">
   <autoFilter ref="A1:F11" xr:uid="{446CC8FA-01E3-483B-8CA2-40098F81BBC1}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{0461F621-E826-4C3D-BDEA-2C1496EF7F1F}" uniqueName="1" name="Customer_ID" queryTableFieldId="1" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{23D3F946-EC33-4F61-A7BA-A9B2C7560B7D}" uniqueName="2" name="Customer_Name" queryTableFieldId="2" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{0428D812-8D8E-417A-A1FB-B4210642DF0C}" uniqueName="3" name="Email_ID" queryTableFieldId="3" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{5842EBB0-F8CF-4E18-8504-17EA3D78B437}" uniqueName="4" name="Phone_Number" queryTableFieldId="4" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{F86DBFA3-86C7-48D5-A1D2-D869943B3366}" uniqueName="5" name="Product_Code" queryTableFieldId="5" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{25487770-C6E2-46F1-A0B0-D5CD99016EC1}" uniqueName="6" name="City" queryTableFieldId="6" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{0461F621-E826-4C3D-BDEA-2C1496EF7F1F}" uniqueName="1" name="Customer_ID" queryTableFieldId="1" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{23D3F946-EC33-4F61-A7BA-A9B2C7560B7D}" uniqueName="2" name="Customer_Name" queryTableFieldId="2" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{0428D812-8D8E-417A-A1FB-B4210642DF0C}" uniqueName="3" name="Email_ID" queryTableFieldId="3" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{5842EBB0-F8CF-4E18-8504-17EA3D78B437}" uniqueName="4" name="Phone_Number" queryTableFieldId="4" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{F86DBFA3-86C7-48D5-A1D2-D869943B3366}" uniqueName="5" name="Product_Code" queryTableFieldId="5" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{25487770-C6E2-46F1-A0B0-D5CD99016EC1}" uniqueName="6" name="City" queryTableFieldId="6" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1021,22 +1005,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="D1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="E1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" s="13" t="s">
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
@@ -1044,263 +1028,263 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="18">
+      <c r="A2" s="14">
         <v>201</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="8">
+      <c r="D2" s="7">
         <v>9876543210</v>
       </c>
-      <c r="E2" s="19" t="s">
+      <c r="E2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="20" t="s">
+      <c r="F2" s="15" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="18">
+      <c r="A3" s="14">
         <v>202</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="7">
         <v>9123456789</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="20" t="s">
+      <c r="F3" s="15" t="s">
         <v>13</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="J3" s="12" t="s">
+      <c r="J3" s="8" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="18">
+      <c r="A4" s="14">
         <v>203</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="7">
         <v>9988776655</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="20" t="s">
+      <c r="F4" s="15" t="s">
         <v>17</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J4" s="13" t="str">
+      <c r="J4" s="9" t="str">
         <f>MID(I4,(FIND("-",I4)+1),2)</f>
         <v>AX</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="18">
+      <c r="A5" s="14">
         <v>204</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="7">
         <v>9012345678</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="F5" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="I5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="J5" s="14" t="str">
+      <c r="J5" s="10" t="str">
         <f>MID(I5,(FIND("-",I5)+1),2)</f>
         <v>BX</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="18">
+      <c r="A6" s="14">
         <v>205</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="7">
         <v>8899776655</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="20" t="s">
+      <c r="F6" s="15" t="s">
         <v>25</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J6" s="13" t="str">
+      <c r="J6" s="9" t="str">
         <f t="shared" ref="J6:J13" si="0">MID(I6,(FIND("-",I6)+1),2)</f>
         <v>CX</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="18">
+      <c r="A7" s="14">
         <v>206</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="7">
         <v>7766554433</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F7" s="20" t="s">
+      <c r="F7" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I7" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="J7" s="14" t="str">
+      <c r="J7" s="10" t="str">
         <f t="shared" si="0"/>
         <v>DX</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="18">
+      <c r="A8" s="14">
         <v>207</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="7">
         <v>6655443322</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="F8" s="20" t="s">
+      <c r="F8" s="15" t="s">
         <v>33</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="J8" s="13" t="str">
+      <c r="J8" s="9" t="str">
         <f t="shared" si="0"/>
         <v>EX</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="18">
+      <c r="A9" s="14">
         <v>208</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="7">
         <v>5544332211</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="F9" s="20" t="s">
+      <c r="F9" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="I9" s="5" t="s">
+      <c r="I9" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="J9" s="14" t="str">
+      <c r="J9" s="10" t="str">
         <f t="shared" si="0"/>
         <v>FX</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="18">
+      <c r="A10" s="14">
         <v>209</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="7">
         <v>4433221100</v>
       </c>
-      <c r="E10" s="19" t="s">
+      <c r="E10" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="F10" s="20" t="s">
+      <c r="F10" s="15" t="s">
         <v>41</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="J10" s="13" t="str">
+      <c r="J10" s="9" t="str">
         <f t="shared" si="0"/>
         <v>GX</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="21">
+      <c r="A11" s="16">
         <v>210</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="23">
+      <c r="D11" s="17">
         <v>3322110099</v>
       </c>
-      <c r="E11" s="22" t="s">
+      <c r="E11" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="F11" s="24" t="s">
+      <c r="F11" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="I11" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="J11" s="14" t="str">
+      <c r="J11" s="10" t="str">
         <f t="shared" si="0"/>
         <v>HX</v>
       </c>
@@ -1309,7 +1293,7 @@
       <c r="I12" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="J12" s="13" t="str">
+      <c r="J12" s="9" t="str">
         <f t="shared" si="0"/>
         <v>IX</v>
       </c>
@@ -1318,19 +1302,19 @@
       <c r="A13" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="I13" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="J13" s="14" t="str">
+      <c r="J13" s="10" t="str">
         <f t="shared" si="0"/>
         <v>JX</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="5" t="s">
         <v>58</v>
       </c>
       <c r="H15" s="1" t="s">
@@ -1338,153 +1322,153 @@
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" s="7">
         <f>LEN(B16)</f>
         <v>12</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C17" s="8">
+      <c r="C17" s="7">
         <f t="shared" ref="C17:C25" si="1">LEN(B17)</f>
         <v>11</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="J17" s="12" t="s">
+      <c r="J17" s="8" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="7">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="I18" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J18" s="13" t="str">
+      <c r="J18" s="9" t="str">
         <f>RIGHT(I18,4)</f>
         <v>1001</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C19" s="7">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="I19" s="5" t="s">
+      <c r="I19" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="J19" s="13" t="str">
+      <c r="J19" s="9" t="str">
         <f t="shared" ref="J19:J27" si="2">RIGHT(I19,4)</f>
         <v>1002</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20" s="7">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
       <c r="I20" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J20" s="13" t="str">
+      <c r="J20" s="9" t="str">
         <f t="shared" si="2"/>
         <v>1003</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C21" s="8">
+      <c r="C21" s="7">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="I21" s="5" t="s">
+      <c r="I21" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="J21" s="13" t="str">
+      <c r="J21" s="9" t="str">
         <f t="shared" si="2"/>
         <v>1004</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="8">
+      <c r="C22" s="7">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="I22" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="J22" s="13" t="str">
+      <c r="J22" s="9" t="str">
         <f t="shared" si="2"/>
         <v>1005</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C23" s="8">
+      <c r="C23" s="7">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="I23" s="5" t="s">
+      <c r="I23" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="J23" s="13" t="str">
+      <c r="J23" s="9" t="str">
         <f t="shared" si="2"/>
         <v>1006</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C24" s="8">
+      <c r="C24" s="7">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
       <c r="I24" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="J24" s="13" t="str">
+      <c r="J24" s="9" t="str">
         <f t="shared" si="2"/>
         <v>1007</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C25" s="8">
+      <c r="C25" s="7">
         <f t="shared" si="1"/>
         <v>14</v>
       </c>
-      <c r="I25" s="5" t="s">
+      <c r="I25" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="J25" s="13" t="str">
+      <c r="J25" s="9" t="str">
         <f t="shared" si="2"/>
         <v>1008</v>
       </c>
@@ -1493,7 +1477,7 @@
       <c r="I26" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="J26" s="13" t="str">
+      <c r="J26" s="9" t="str">
         <f t="shared" si="2"/>
         <v>1009</v>
       </c>
@@ -1502,19 +1486,19 @@
       <c r="A27" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I27" s="5" t="s">
+      <c r="I27" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="J27" s="13" t="str">
+      <c r="J27" s="9" t="str">
         <f t="shared" si="2"/>
         <v>1010</v>
       </c>
     </row>
     <row r="29" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="5" t="s">
         <v>58</v>
       </c>
       <c r="H29" s="1" t="s">
@@ -1525,181 +1509,181 @@
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C30" s="8">
-        <f>LEN(C2)</f>
+      <c r="C30" s="7">
+        <f t="shared" ref="C30:C39" si="3">LEN(C2)</f>
         <v>22</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B31" s="9" t="s">
+      <c r="B31" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C31" s="8">
-        <f>LEN(C3)</f>
+      <c r="C31" s="7">
+        <f t="shared" si="3"/>
         <v>21</v>
       </c>
       <c r="I31" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="J31" s="6" t="s">
+      <c r="J31" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K31" s="12" t="s">
+      <c r="K31" s="8" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B32" s="7" t="s">
+      <c r="B32" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C32" s="8">
-        <f>LEN(C4)</f>
+      <c r="C32" s="7">
+        <f t="shared" si="3"/>
         <v>22</v>
       </c>
       <c r="I32" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="J32" s="7" t="s">
+      <c r="J32" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="K32" s="13" t="str">
+      <c r="K32" s="9" t="str">
         <f>LEFT(J32,(FIND(".",J32)-1))</f>
         <v>rahul</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B33" s="9" t="s">
+      <c r="B33" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C33" s="8">
-        <f>LEN(C5)</f>
+      <c r="C33" s="7">
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="I33" s="5" t="s">
+      <c r="I33" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J33" s="9" t="s">
+      <c r="J33" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="K33" s="13" t="str">
-        <f t="shared" ref="K33:K41" si="3">LEFT(J33,(FIND(".",J33)-1))</f>
+      <c r="K33" s="9" t="str">
+        <f t="shared" ref="K33:K41" si="4">LEFT(J33,(FIND(".",J33)-1))</f>
         <v>priya</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B34" s="7" t="s">
+      <c r="B34" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C34" s="8">
-        <f>LEN(C6)</f>
+      <c r="C34" s="7">
+        <f t="shared" si="3"/>
         <v>21</v>
       </c>
       <c r="I34" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J34" s="7" t="s">
+      <c r="J34" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="K34" s="13" t="str">
+      <c r="K34" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v>anil</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B35" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C35" s="7">
         <f t="shared" si="3"/>
-        <v>anil</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B35" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="C35" s="8">
-        <f>LEN(C7)</f>
         <v>20</v>
       </c>
-      <c r="I35" s="5" t="s">
+      <c r="I35" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="J35" s="9" t="s">
+      <c r="J35" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="K35" s="13" t="str">
+      <c r="K35" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v>sneha</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B36" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C36" s="7">
         <f t="shared" si="3"/>
-        <v>sneha</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B36" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="C36" s="8">
-        <f>LEN(C8)</f>
         <v>22</v>
       </c>
       <c r="I36" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J36" s="7" t="s">
+      <c r="J36" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="K36" s="13" t="str">
+      <c r="K36" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v>rohit</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B37" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C37" s="7">
         <f t="shared" si="3"/>
-        <v>rohit</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B37" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="C37" s="8">
-        <f>LEN(C9)</f>
         <v>22</v>
       </c>
-      <c r="I37" s="5" t="s">
+      <c r="I37" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="J37" s="9" t="s">
+      <c r="J37" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="K37" s="13" t="str">
+      <c r="K37" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v>neha</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B38" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C38" s="7">
         <f t="shared" si="3"/>
-        <v>neha</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B38" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C38" s="8">
-        <f>LEN(C10)</f>
         <v>21</v>
       </c>
       <c r="I38" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="J38" s="7" t="s">
+      <c r="J38" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="K38" s="13" t="str">
+      <c r="K38" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v>amit</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B39" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C39" s="7">
         <f t="shared" si="3"/>
-        <v>amit</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B39" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C39" s="8">
-        <f>LEN(C11)</f>
         <v>24</v>
       </c>
-      <c r="I39" s="5" t="s">
+      <c r="I39" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="J39" s="9" t="s">
+      <c r="J39" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="K39" s="13" t="str">
-        <f t="shared" si="3"/>
+      <c r="K39" s="9" t="str">
+        <f t="shared" si="4"/>
         <v>kavita</v>
       </c>
     </row>
@@ -1707,11 +1691,11 @@
       <c r="I40" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="J40" s="7" t="s">
+      <c r="J40" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="K40" s="13" t="str">
-        <f t="shared" si="3"/>
+      <c r="K40" s="9" t="str">
+        <f t="shared" si="4"/>
         <v>suresh</v>
       </c>
     </row>
@@ -1719,14 +1703,14 @@
       <c r="A41" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I41" s="5" t="s">
+      <c r="I41" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="J41" s="9" t="s">
+      <c r="J41" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="K41" s="13" t="str">
-        <f t="shared" si="3"/>
+      <c r="K41" s="9" t="str">
+        <f t="shared" si="4"/>
         <v>pooja</v>
       </c>
     </row>
@@ -1751,17 +1735,17 @@
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B45" s="5" t="s">
+      <c r="B45" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C45" s="4" t="str">
-        <f t="shared" ref="C45:C53" si="4">LEFT(B45,5)</f>
+        <f t="shared" ref="C45:C53" si="5">LEFT(B45,5)</f>
         <v>Priya</v>
       </c>
-      <c r="J45" s="6" t="s">
+      <c r="J45" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K45" s="25" t="s">
+      <c r="K45" s="19" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1770,30 +1754,30 @@
         <v>14</v>
       </c>
       <c r="C46" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">Anil </v>
       </c>
-      <c r="J46" s="7" t="s">
+      <c r="J46" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="K46" s="26" t="str">
+      <c r="K46" s="20" t="str">
         <f>MID(J46,FIND("@",J46),20)</f>
         <v>@gmail.com</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B47" s="5" t="s">
+      <c r="B47" s="4" t="s">
         <v>18</v>
       </c>
       <c r="C47" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>Sneha</v>
       </c>
-      <c r="J47" s="9" t="s">
+      <c r="J47" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="K47" s="26" t="str">
-        <f t="shared" ref="K47:K55" si="5">MID(J47,FIND("@",J47),20)</f>
+      <c r="K47" s="20" t="str">
+        <f t="shared" ref="K47:K55" si="6">MID(J47,FIND("@",J47),20)</f>
         <v>@yahoo.com</v>
       </c>
     </row>
@@ -1802,30 +1786,30 @@
         <v>22</v>
       </c>
       <c r="C48" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>Rohit</v>
       </c>
-      <c r="J48" s="7" t="s">
+      <c r="J48" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="K48" s="26" t="str">
+      <c r="K48" s="20" t="str">
+        <f t="shared" si="6"/>
+        <v>@outlook.com</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B49" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C49" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>@outlook.com</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B49" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C49" s="4" t="str">
-        <f t="shared" si="4"/>
         <v xml:space="preserve">Neha </v>
       </c>
-      <c r="J49" s="9" t="s">
+      <c r="J49" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="K49" s="26" t="str">
-        <f t="shared" si="5"/>
+      <c r="K49" s="20" t="str">
+        <f t="shared" si="6"/>
         <v>@gmail.com</v>
       </c>
     </row>
@@ -1834,30 +1818,30 @@
         <v>30</v>
       </c>
       <c r="C50" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">Amit </v>
       </c>
-      <c r="J50" s="7" t="s">
+      <c r="J50" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="K50" s="26" t="str">
+      <c r="K50" s="20" t="str">
+        <f t="shared" si="6"/>
+        <v>@yahoo.com</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B51" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C51" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>@yahoo.com</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B51" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C51" s="4" t="str">
-        <f t="shared" si="4"/>
         <v>Kavit</v>
       </c>
-      <c r="J51" s="9" t="s">
+      <c r="J51" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="K51" s="26" t="str">
-        <f t="shared" si="5"/>
+      <c r="K51" s="20" t="str">
+        <f t="shared" si="6"/>
         <v>@gmail.com</v>
       </c>
     </row>
@@ -1866,39 +1850,39 @@
         <v>38</v>
       </c>
       <c r="C52" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>Sures</v>
       </c>
-      <c r="J52" s="7" t="s">
+      <c r="J52" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="K52" s="26" t="str">
+      <c r="K52" s="20" t="str">
+        <f t="shared" si="6"/>
+        <v>@outlook.com</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B53" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C53" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>@outlook.com</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B53" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C53" s="4" t="str">
-        <f t="shared" si="4"/>
         <v>Pooja</v>
       </c>
-      <c r="J53" s="9" t="s">
+      <c r="J53" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="K53" s="26" t="str">
-        <f t="shared" si="5"/>
+      <c r="K53" s="20" t="str">
+        <f t="shared" si="6"/>
         <v>@gmail.com</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="J54" s="7" t="s">
+      <c r="J54" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="K54" s="26" t="str">
-        <f t="shared" si="5"/>
+      <c r="K54" s="20" t="str">
+        <f t="shared" si="6"/>
         <v>@yahoo.com</v>
       </c>
     </row>
@@ -1906,19 +1890,19 @@
       <c r="A55" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="J55" s="9" t="s">
+      <c r="J55" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="K55" s="26" t="str">
-        <f t="shared" si="5"/>
+      <c r="K55" s="20" t="str">
+        <f t="shared" si="6"/>
         <v>@gmail.com</v>
       </c>
     </row>
     <row r="57" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B57" s="6" t="s">
+      <c r="B57" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C57" s="6" t="s">
+      <c r="C57" s="5" t="s">
         <v>60</v>
       </c>
       <c r="H57" s="1" t="s">
@@ -1926,163 +1910,163 @@
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B58" s="10">
+      <c r="B58" s="6">
         <v>9876543210</v>
       </c>
-      <c r="C58" s="10" t="str">
+      <c r="C58" s="6" t="str">
         <f>RIGHT(B58,4)</f>
         <v>3210</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B59" s="11">
+      <c r="B59" s="7">
         <v>9123456789</v>
       </c>
-      <c r="C59" s="10" t="str">
-        <f t="shared" ref="C59:C67" si="6">RIGHT(B59,4)</f>
+      <c r="C59" s="6" t="str">
+        <f t="shared" ref="C59:C67" si="7">RIGHT(B59,4)</f>
         <v>6789</v>
       </c>
-      <c r="I59" s="6" t="s">
+      <c r="I59" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="J59" s="6" t="s">
+      <c r="J59" s="5" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B60" s="10">
+      <c r="B60" s="6">
         <v>9988776655</v>
       </c>
-      <c r="C60" s="10" t="str">
-        <f t="shared" si="6"/>
+      <c r="C60" s="6" t="str">
+        <f t="shared" si="7"/>
         <v>6655</v>
       </c>
-      <c r="I60" s="7" t="s">
+      <c r="I60" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J60" s="7">
+      <c r="J60" s="6">
         <f>LEN(I60)</f>
         <v>11</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B61" s="11">
+      <c r="B61" s="7">
         <v>9012345678</v>
       </c>
-      <c r="C61" s="10" t="str">
-        <f t="shared" si="6"/>
+      <c r="C61" s="6" t="str">
+        <f t="shared" si="7"/>
         <v>5678</v>
       </c>
-      <c r="I61" s="9" t="s">
+      <c r="I61" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="J61" s="7">
-        <f t="shared" ref="J61:J69" si="7">LEN(I61)</f>
+      <c r="J61" s="6">
+        <f t="shared" ref="J61:J69" si="8">LEN(I61)</f>
         <v>11</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B62" s="10">
+      <c r="B62" s="6">
         <v>8899776655</v>
       </c>
-      <c r="C62" s="10" t="str">
-        <f t="shared" si="6"/>
+      <c r="C62" s="6" t="str">
+        <f t="shared" si="7"/>
         <v>6655</v>
       </c>
-      <c r="I62" s="7" t="s">
+      <c r="I62" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="J62" s="7">
+      <c r="J62" s="6">
+        <f t="shared" si="8"/>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B63" s="7">
+        <v>7766554433</v>
+      </c>
+      <c r="C63" s="6" t="str">
         <f t="shared" si="7"/>
+        <v>4433</v>
+      </c>
+      <c r="I63" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J63" s="6">
+        <f t="shared" si="8"/>
         <v>11</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B63" s="11">
-        <v>7766554433</v>
-      </c>
-      <c r="C63" s="10" t="str">
-        <f t="shared" si="6"/>
-        <v>4433</v>
-      </c>
-      <c r="I63" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="J63" s="7">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B64" s="6">
+        <v>6655443322</v>
+      </c>
+      <c r="C64" s="6" t="str">
         <f t="shared" si="7"/>
+        <v>3322</v>
+      </c>
+      <c r="I64" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J64" s="6">
+        <f t="shared" si="8"/>
         <v>11</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B64" s="10">
-        <v>6655443322</v>
-      </c>
-      <c r="C64" s="10" t="str">
-        <f t="shared" si="6"/>
-        <v>3322</v>
-      </c>
-      <c r="I64" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="J64" s="7">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B65" s="7">
+        <v>5544332211</v>
+      </c>
+      <c r="C65" s="6" t="str">
         <f t="shared" si="7"/>
+        <v>2211</v>
+      </c>
+      <c r="I65" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="J65" s="6">
+        <f t="shared" si="8"/>
         <v>11</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B65" s="11">
-        <v>5544332211</v>
-      </c>
-      <c r="C65" s="10" t="str">
-        <f t="shared" si="6"/>
-        <v>2211</v>
-      </c>
-      <c r="I65" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J65" s="7">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B66" s="6">
+        <v>4433221100</v>
+      </c>
+      <c r="C66" s="6" t="str">
         <f t="shared" si="7"/>
+        <v>1100</v>
+      </c>
+      <c r="I66" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="J66" s="6">
+        <f t="shared" si="8"/>
         <v>11</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B66" s="10">
-        <v>4433221100</v>
-      </c>
-      <c r="C66" s="10" t="str">
-        <f t="shared" si="6"/>
-        <v>1100</v>
-      </c>
-      <c r="I66" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="J66" s="7">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B67" s="7">
+        <v>3322110099</v>
+      </c>
+      <c r="C67" s="6" t="str">
         <f t="shared" si="7"/>
+        <v>0099</v>
+      </c>
+      <c r="I67" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="J67" s="6">
+        <f t="shared" si="8"/>
         <v>11</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B67" s="11">
-        <v>3322110099</v>
-      </c>
-      <c r="C67" s="10" t="str">
-        <f t="shared" si="6"/>
-        <v>0099</v>
-      </c>
-      <c r="I67" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="J67" s="7">
-        <f t="shared" si="7"/>
-        <v>11</v>
-      </c>
-    </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="I68" s="7" t="s">
+      <c r="I68" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="J68" s="7">
-        <f t="shared" si="7"/>
+      <c r="J68" s="6">
+        <f t="shared" si="8"/>
         <v>11</v>
       </c>
     </row>
@@ -2090,11 +2074,11 @@
       <c r="A69" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="I69" s="9" t="s">
+      <c r="I69" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="J69" s="7">
-        <f t="shared" si="7"/>
+      <c r="J69" s="6">
+        <f t="shared" si="8"/>
         <v>11</v>
       </c>
     </row>
@@ -2119,11 +2103,11 @@
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B73" s="5" t="s">
+      <c r="B73" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C73" s="3" t="str">
-        <f t="shared" ref="C73:C81" si="8">LEFT(B73,3)</f>
+        <f t="shared" ref="C73:C81" si="9">LEFT(B73,3)</f>
         <v>PRD</v>
       </c>
     </row>
@@ -2132,28 +2116,28 @@
         <v>16</v>
       </c>
       <c r="C74" s="3" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>PRD</v>
       </c>
-      <c r="I74" s="25" t="s">
+      <c r="I74" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="J74" s="25" t="s">
+      <c r="J74" s="19" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B75" s="5" t="s">
+      <c r="B75" s="4" t="s">
         <v>20</v>
       </c>
       <c r="C75" s="3" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>PRD</v>
       </c>
-      <c r="I75" s="26" t="s">
+      <c r="I75" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="J75" s="26" t="str">
+      <c r="J75" s="20" t="str">
         <f>LEFT(I75,1)</f>
         <v>M</v>
       </c>
@@ -2163,30 +2147,30 @@
         <v>24</v>
       </c>
       <c r="C76" s="3" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>PRD</v>
       </c>
-      <c r="I76" s="27" t="s">
+      <c r="I76" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="J76" s="26" t="str">
-        <f t="shared" ref="J76:J84" si="9">LEFT(I76,1)</f>
+      <c r="J76" s="20" t="str">
+        <f t="shared" ref="J76:J84" si="10">LEFT(I76,1)</f>
         <v>A</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B77" s="5" t="s">
+      <c r="B77" s="4" t="s">
         <v>28</v>
       </c>
       <c r="C77" s="3" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>PRD</v>
       </c>
-      <c r="I77" s="26" t="s">
+      <c r="I77" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="J77" s="26" t="str">
-        <f t="shared" si="9"/>
+      <c r="J77" s="20" t="str">
+        <f t="shared" si="10"/>
         <v>D</v>
       </c>
     </row>
@@ -2195,30 +2179,30 @@
         <v>32</v>
       </c>
       <c r="C78" s="3" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>PRD</v>
       </c>
-      <c r="I78" s="27" t="s">
+      <c r="I78" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="J78" s="26" t="str">
+      <c r="J78" s="20" t="str">
+        <f t="shared" si="10"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B79" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C79" s="3" t="str">
         <f t="shared" si="9"/>
-        <v>C</v>
-      </c>
-    </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B79" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C79" s="3" t="str">
-        <f t="shared" si="8"/>
         <v>PRD</v>
       </c>
-      <c r="I79" s="26" t="s">
+      <c r="I79" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="J79" s="26" t="str">
-        <f t="shared" si="9"/>
+      <c r="J79" s="20" t="str">
+        <f t="shared" si="10"/>
         <v>P</v>
       </c>
     </row>
@@ -2227,57 +2211,57 @@
         <v>40</v>
       </c>
       <c r="C80" s="3" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>PRD</v>
       </c>
-      <c r="I80" s="27" t="s">
+      <c r="I80" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="J80" s="26" t="str">
+      <c r="J80" s="20" t="str">
+        <f t="shared" si="10"/>
+        <v>J</v>
+      </c>
+    </row>
+    <row r="81" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B81" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C81" s="3" t="str">
         <f t="shared" si="9"/>
-        <v>J</v>
-      </c>
-    </row>
-    <row r="81" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B81" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="C81" s="3" t="str">
-        <f t="shared" si="8"/>
         <v>PRD</v>
       </c>
-      <c r="I81" s="26" t="s">
+      <c r="I81" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="J81" s="26" t="str">
-        <f t="shared" si="9"/>
+      <c r="J81" s="20" t="str">
+        <f t="shared" si="10"/>
         <v>B</v>
       </c>
     </row>
     <row r="82" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="I82" s="27" t="s">
+      <c r="I82" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="J82" s="26" t="str">
-        <f t="shared" si="9"/>
+      <c r="J82" s="20" t="str">
+        <f t="shared" si="10"/>
         <v>I</v>
       </c>
     </row>
     <row r="83" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="I83" s="26" t="s">
+      <c r="I83" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="J83" s="26" t="str">
-        <f t="shared" si="9"/>
+      <c r="J83" s="20" t="str">
+        <f t="shared" si="10"/>
         <v>K</v>
       </c>
     </row>
     <row r="84" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="I84" s="27" t="s">
+      <c r="I84" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="J84" s="26" t="str">
-        <f t="shared" si="9"/>
+      <c r="J84" s="20" t="str">
+        <f t="shared" si="10"/>
         <v>N</v>
       </c>
     </row>
@@ -2287,100 +2271,100 @@
       </c>
     </row>
     <row r="88" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="I88" s="6" t="s">
+      <c r="I88" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="J88" s="6" t="s">
+      <c r="J88" s="5" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="89" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="I89" s="7" t="s">
+      <c r="I89" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="J89" s="7" t="str">
+      <c r="J89" s="6" t="str">
         <f>RIGHT(I89,2)</f>
         <v>ai</v>
       </c>
     </row>
     <row r="90" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="I90" s="9" t="s">
+      <c r="I90" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="J90" s="7" t="str">
-        <f t="shared" ref="J90:J98" si="10">RIGHT(I90,2)</f>
+      <c r="J90" s="6" t="str">
+        <f t="shared" ref="J90:J98" si="11">RIGHT(I90,2)</f>
         <v>ad</v>
       </c>
     </row>
     <row r="91" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="I91" s="7" t="s">
+      <c r="I91" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="J91" s="7" t="str">
-        <f t="shared" si="10"/>
+      <c r="J91" s="6" t="str">
+        <f t="shared" si="11"/>
         <v>hi</v>
       </c>
     </row>
     <row r="92" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="I92" s="9" t="s">
+      <c r="I92" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="J92" s="7" t="str">
-        <f t="shared" si="10"/>
+      <c r="J92" s="6" t="str">
+        <f t="shared" si="11"/>
         <v>ai</v>
       </c>
     </row>
     <row r="93" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="I93" s="7" t="s">
+      <c r="I93" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="J93" s="7" t="str">
-        <f t="shared" si="10"/>
+      <c r="J93" s="6" t="str">
+        <f t="shared" si="11"/>
         <v>ne</v>
       </c>
     </row>
     <row r="94" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="I94" s="9" t="s">
+      <c r="I94" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="J94" s="7" t="str">
-        <f t="shared" si="10"/>
+      <c r="J94" s="6" t="str">
+        <f t="shared" si="11"/>
         <v>ur</v>
       </c>
     </row>
     <row r="95" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="I95" s="7" t="s">
+      <c r="I95" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="J95" s="7" t="str">
-        <f t="shared" si="10"/>
+      <c r="J95" s="6" t="str">
+        <f t="shared" si="11"/>
         <v>al</v>
       </c>
     </row>
     <row r="96" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="I96" s="9" t="s">
+      <c r="I96" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="J96" s="7" t="str">
-        <f t="shared" si="10"/>
+      <c r="J96" s="6" t="str">
+        <f t="shared" si="11"/>
         <v>re</v>
       </c>
     </row>
     <row r="97" spans="9:10" x14ac:dyDescent="0.3">
-      <c r="I97" s="7" t="s">
+      <c r="I97" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="J97" s="7" t="str">
-        <f t="shared" si="10"/>
+      <c r="J97" s="6" t="str">
+        <f t="shared" si="11"/>
         <v>hi</v>
       </c>
     </row>
     <row r="98" spans="9:10" x14ac:dyDescent="0.3">
-      <c r="I98" s="9" t="s">
+      <c r="I98" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="J98" s="7" t="str">
-        <f t="shared" si="10"/>
+      <c r="J98" s="6" t="str">
+        <f t="shared" si="11"/>
         <v>ik</v>
       </c>
     </row>

</xml_diff>